<commit_message>
fix: resolve SIRET collision in tests and PostgreSQL-compatible global search
- Change example import SIRETs to avoid collision with test fixtures
- Rewrite ClientSearch to use EXISTS subqueries instead of DISTINCT + JOIN
  (fixes PostgreSQL "ORDER BY must appear in select list" error)
</commit_message>
<xml_diff>
--- a/public/examples/import_clients_exemple.xlsx
+++ b/public/examples/import_clients_exemple.xlsx
@@ -421,7 +421,7 @@
         <v>3</v>
       </c>
       <c r="B2">
-        <v>12345678901234</v>
+        <v>55566677788899</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
@@ -432,7 +432,7 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>98765432109876</v>
+        <v>99988877766655</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -443,7 +443,7 @@
         <v>7</v>
       </c>
       <c r="B4">
-        <v>11122233344455</v>
+        <v>44433322211100</v>
       </c>
       <c r="C4" t="s">
         <v>8</v>

</xml_diff>